<commit_message>
Refactor doctor department classifications for improved accuracy and consistency across specialties
</commit_message>
<xml_diff>
--- a/MendSure_Departments_Doctors_Hospitals.xlsx
+++ b/MendSure_Departments_Doctors_Hospitals.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d500d5bbca9d05a/Documents/Mendsure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{C40ADF73-3C2A-4183-8D64-1E8B5B5BB951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67E34F8B-1F63-484F-8B38-1A0262404FC5}"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="8_{C40ADF73-3C2A-4183-8D64-1E8B5B5BB951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BA7CF4B-997D-4089-9D99-614716F1BF92}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="991" uniqueCount="307">
   <si>
     <t>MendSure — Specialists, Departments, Doctors &amp; Hospitals</t>
   </si>
@@ -866,36 +866,18 @@
     <t>Urology Care</t>
   </si>
   <si>
-    <t>Nephrology &amp; Kidney Transplant Medicine</t>
-  </si>
-  <si>
-    <t>Urology and Kidney Transplant Surgery</t>
-  </si>
-  <si>
     <t xml:space="preserve">Neurosurgery </t>
   </si>
   <si>
-    <t>Oncology Gynaecology Surgery</t>
-  </si>
-  <si>
     <t>Oncology Radiation</t>
   </si>
   <si>
-    <t>ENT Oncology Surgery</t>
-  </si>
-  <si>
     <t>Oncology Surgery</t>
   </si>
   <si>
-    <t>Orthopaedic Oncology Surgery</t>
-  </si>
-  <si>
     <t xml:space="preserve">Haematology </t>
   </si>
   <si>
-    <t xml:space="preserve">Pediatric Haematology </t>
-  </si>
-  <si>
     <t>Pediatric Care</t>
   </si>
   <si>
@@ -903,13 +885,76 @@
   </si>
   <si>
     <t>Lung Transplant Surgery</t>
+  </si>
+  <si>
+    <t>Neuro Surgery</t>
+  </si>
+  <si>
+    <t>Vascular Surgery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cardiology </t>
+  </si>
+  <si>
+    <t>ENT Surgery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gastroenterology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urology </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oncology Surgery </t>
+  </si>
+  <si>
+    <t>Kidney Transplant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVF and Infertility </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gynecology and Obestrics </t>
+  </si>
+  <si>
+    <t>Bariatic Surgery</t>
+  </si>
+  <si>
+    <t>Dermatology</t>
+  </si>
+  <si>
+    <t>Endocrinology</t>
+  </si>
+  <si>
+    <t>Dental Treatment</t>
+  </si>
+  <si>
+    <t>Eye Treatment and Surgery</t>
+  </si>
+  <si>
+    <t>Pulmonology</t>
+  </si>
+  <si>
+    <t>Cosmetic and Plastic Surgery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulmonology </t>
+  </si>
+  <si>
+    <t>Hepatology</t>
+  </si>
+  <si>
+    <t>Nephrology and Urology ke doctors hi liver transplant ke hain</t>
+  </si>
+  <si>
+    <t>Hepatology ke doctor Liver transplant ke hain</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -939,6 +984,19 @@
       <color rgb="FF808080"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -966,7 +1024,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -989,11 +1047,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1043,6 +1112,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1345,11 +1434,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:J145"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="26.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
@@ -1359,7 +1448,7 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
@@ -1372,7 +1461,7 @@
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
     </row>
-    <row r="3" spans="1:9" ht="28" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="28" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1401,7 +1490,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -1409,7 +1498,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>288</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>12</v>
@@ -1430,7 +1519,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <f>A4+1</f>
         <v>2</v>
@@ -1438,8 +1527,8 @@
       <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>11</v>
+      <c r="C5" s="3" t="s">
+        <v>288</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>17</v>
@@ -1460,7 +1549,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <f t="shared" ref="A6:A69" si="0">A5+1</f>
         <v>3</v>
@@ -1469,7 +1558,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>11</v>
+        <v>288</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>19</v>
@@ -1490,7 +1579,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1498,8 +1587,8 @@
       <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>43</v>
+      <c r="C7" s="3" t="s">
+        <v>288</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>44</v>
@@ -1519,8 +1608,11 @@
       <c r="I7" s="4">
         <v>35</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J7" s="19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1528,8 +1620,8 @@
       <c r="B8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>22</v>
+      <c r="C8" s="3" t="s">
+        <v>288</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>23</v>
@@ -1550,7 +1642,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1558,8 +1650,8 @@
       <c r="B9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>22</v>
+      <c r="C9" s="3" t="s">
+        <v>288</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>27</v>
@@ -1580,7 +1672,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1588,8 +1680,8 @@
       <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>22</v>
+      <c r="C10" s="3" t="s">
+        <v>288</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>29</v>
@@ -1610,7 +1702,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1619,7 +1711,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>22</v>
+        <v>288</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>33</v>
@@ -1640,7 +1732,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1648,8 +1740,8 @@
       <c r="B12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>22</v>
+      <c r="C12" s="3" t="s">
+        <v>288</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>36</v>
@@ -1670,7 +1762,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1679,7 +1771,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>22</v>
+        <v>288</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>37</v>
@@ -1700,7 +1792,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1708,8 +1800,8 @@
       <c r="B14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>22</v>
+      <c r="C14" s="3" t="s">
+        <v>288</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>39</v>
@@ -1730,7 +1822,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1739,7 +1831,7 @@
         <v>10</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>22</v>
+        <v>288</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>41</v>
@@ -1760,7 +1852,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1769,7 +1861,7 @@
         <v>10</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>45</v>
+        <v>288</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>46</v>
@@ -2488,8 +2580,8 @@
       <c r="B40" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>81</v>
+      <c r="C40" s="25" t="s">
+        <v>302</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>82</v>
@@ -2518,8 +2610,8 @@
       <c r="B41" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="5" t="s">
-        <v>81</v>
+      <c r="C41" s="25" t="s">
+        <v>302</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>84</v>
@@ -2549,7 +2641,7 @@
         <v>86</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>89</v>
+        <v>289</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>88</v>
@@ -2579,7 +2671,7 @@
         <v>86</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>89</v>
+        <v>289</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>90</v>
@@ -2609,7 +2701,7 @@
         <v>91</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>92</v>
+        <v>290</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>93</v>
@@ -2638,8 +2730,8 @@
       <c r="B45" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C45" s="5" t="s">
-        <v>92</v>
+      <c r="C45" s="3" t="s">
+        <v>290</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>95</v>
@@ -2669,7 +2761,7 @@
         <v>97</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>98</v>
+        <v>290</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>99</v>
@@ -2698,8 +2790,8 @@
       <c r="B47" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C47" s="5" t="s">
-        <v>98</v>
+      <c r="C47" s="3" t="s">
+        <v>290</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>101</v>
@@ -2729,7 +2821,7 @@
         <v>151</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>105</v>
@@ -2758,8 +2850,8 @@
       <c r="B49" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C49" s="3" t="s">
-        <v>109</v>
+      <c r="C49" s="22" t="s">
+        <v>106</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>107</v>
@@ -2788,8 +2880,8 @@
       <c r="B50" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C50" s="3" t="s">
-        <v>109</v>
+      <c r="C50" s="22" t="s">
+        <v>106</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>110</v>
@@ -2818,8 +2910,8 @@
       <c r="B51" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C51" s="3" t="s">
-        <v>109</v>
+      <c r="C51" s="22" t="s">
+        <v>106</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>112</v>
@@ -2908,8 +3000,8 @@
       <c r="B54" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C54" s="3" t="s">
-        <v>118</v>
+      <c r="C54" s="25" t="s">
+        <v>303</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>119</v>
@@ -2939,7 +3031,7 @@
         <v>277</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>123</v>
@@ -2968,8 +3060,8 @@
       <c r="B56" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="C56" s="3" t="s">
-        <v>279</v>
+      <c r="C56" s="7" t="s">
+        <v>277</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>124</v>
@@ -2998,8 +3090,8 @@
       <c r="B57" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="C57" s="5" t="s">
-        <v>279</v>
+      <c r="C57" s="7" t="s">
+        <v>277</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>125</v>
@@ -3029,7 +3121,7 @@
         <v>278</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>127</v>
@@ -3059,7 +3151,7 @@
         <v>278</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>129</v>
@@ -3089,7 +3181,7 @@
         <v>278</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="D60" s="7" t="s">
         <v>132</v>
@@ -3119,7 +3211,7 @@
         <v>278</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>133</v>
@@ -3149,7 +3241,7 @@
         <v>278</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>134</v>
@@ -3176,10 +3268,10 @@
         <v>60</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>136</v>
+        <v>286</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>137</v>
@@ -3206,10 +3298,10 @@
         <v>61</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="C64" s="7" t="s">
-        <v>135</v>
+        <v>279</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>286</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>139</v>
@@ -3236,10 +3328,10 @@
         <v>62</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="C65" s="7" t="s">
-        <v>135</v>
+        <v>279</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>286</v>
       </c>
       <c r="D65" s="7" t="s">
         <v>140</v>
@@ -3266,10 +3358,10 @@
         <v>63</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="C66" s="7" t="s">
-        <v>135</v>
+        <v>279</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>286</v>
       </c>
       <c r="D66" s="7" t="s">
         <v>141</v>
@@ -3296,10 +3388,10 @@
         <v>64</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>135</v>
+        <v>286</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>142</v>
@@ -3326,10 +3418,10 @@
         <v>65</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>135</v>
+        <v>279</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>286</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>143</v>
@@ -3356,7 +3448,7 @@
         <v>66</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C69" s="5" t="s">
         <v>145</v>
@@ -3386,7 +3478,7 @@
         <v>67</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C70" s="5" t="s">
         <v>145</v>
@@ -3419,7 +3511,7 @@
         <v>151</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="D71" s="7" t="s">
         <v>153</v>
@@ -3449,7 +3541,7 @@
         <v>151</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>154</v>
@@ -3478,8 +3570,8 @@
       <c r="B73" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C73" s="5" t="s">
-        <v>288</v>
+      <c r="C73" s="3" t="s">
+        <v>282</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>156</v>
@@ -3598,8 +3690,8 @@
       <c r="B77" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C77" s="5" t="s">
-        <v>162</v>
+      <c r="C77" s="7" t="s">
+        <v>157</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>163</v>
@@ -3629,7 +3721,7 @@
         <v>151</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>166</v>
@@ -3659,7 +3751,7 @@
         <v>151</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>168</v>
@@ -3689,7 +3781,7 @@
         <v>151</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>170</v>
@@ -3718,8 +3810,8 @@
       <c r="B81" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C81" s="5" t="s">
-        <v>284</v>
+      <c r="C81" s="7" t="s">
+        <v>292</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>172</v>
@@ -3749,7 +3841,7 @@
         <v>151</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="D82" s="7" t="s">
         <v>173</v>
@@ -3779,7 +3871,7 @@
         <v>151</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="D83" s="7" t="s">
         <v>174</v>
@@ -3809,7 +3901,7 @@
         <v>151</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D84" s="7" t="s">
         <v>176</v>
@@ -3839,7 +3931,7 @@
         <v>151</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>177</v>
@@ -3869,7 +3961,7 @@
         <v>151</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D86" s="7" t="s">
         <v>179</v>
@@ -3898,8 +3990,8 @@
       <c r="B87" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C87" s="5" t="s">
-        <v>286</v>
+      <c r="C87" s="7" t="s">
+        <v>281</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>183</v>
@@ -3928,7 +4020,7 @@
       <c r="B88" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="C88" s="7" t="s">
+      <c r="C88" s="26" t="s">
         <v>186</v>
       </c>
       <c r="D88" s="7" t="s">
@@ -4288,8 +4380,8 @@
       <c r="B100" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C100" s="3" t="s">
-        <v>204</v>
+      <c r="C100" s="21" t="s">
+        <v>284</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>205</v>
@@ -4316,10 +4408,10 @@
         <v>98</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>208</v>
@@ -4349,7 +4441,7 @@
         <v>210</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>211</v>
+        <v>287</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>212</v>
@@ -4378,8 +4470,8 @@
       <c r="B103" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="C103" s="5" t="s">
-        <v>211</v>
+      <c r="C103" s="3" t="s">
+        <v>287</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>213</v>
@@ -4439,7 +4531,7 @@
         <v>217</v>
       </c>
       <c r="C105" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D105" s="7" t="s">
         <v>219</v>
@@ -4469,7 +4561,7 @@
         <v>217</v>
       </c>
       <c r="C106" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D106" s="7" t="s">
         <v>221</v>
@@ -4502,6 +4594,334 @@
       <c r="G108" s="16"/>
       <c r="H108" s="16"/>
       <c r="I108" s="16"/>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A113" s="23">
+        <v>1</v>
+      </c>
+      <c r="B113" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C113" s="20"/>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A114" s="23">
+        <f>A113+1</f>
+        <v>2</v>
+      </c>
+      <c r="B114" s="24" t="s">
+        <v>276</v>
+      </c>
+      <c r="C114" s="21"/>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A115" s="23">
+        <f t="shared" ref="A115:A145" si="2">A114+1</f>
+        <v>3</v>
+      </c>
+      <c r="B115" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="C115" s="21"/>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A116" s="23">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="B116" s="24" t="s">
+        <v>275</v>
+      </c>
+      <c r="C116" s="21"/>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A117" s="23">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="B117" s="24" t="s">
+        <v>302</v>
+      </c>
+      <c r="C117" s="21"/>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A118" s="23">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="B118" s="24" t="s">
+        <v>289</v>
+      </c>
+      <c r="C118" s="21"/>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A119" s="23">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="B119" s="24" t="s">
+        <v>290</v>
+      </c>
+      <c r="C119" s="21"/>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A120" s="23">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="B120" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="C120" s="21"/>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A121" s="23">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="B121" s="24" t="s">
+        <v>277</v>
+      </c>
+      <c r="C121" s="21"/>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A122" s="23">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="B122" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="C122" s="21"/>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A123" s="23">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="B123" s="24" t="s">
+        <v>286</v>
+      </c>
+      <c r="C123" s="21"/>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A124" s="23">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="B124" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="C124" s="21"/>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A125" s="23">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="B125" s="24" t="s">
+        <v>282</v>
+      </c>
+      <c r="C125" s="21"/>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A126" s="23">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="B126" s="24" t="s">
+        <v>157</v>
+      </c>
+      <c r="C126" s="21"/>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A127" s="23">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="B127" s="24" t="s">
+        <v>281</v>
+      </c>
+      <c r="C127" s="21"/>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A128" s="23">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="B128" s="24" t="s">
+        <v>280</v>
+      </c>
+      <c r="C128" s="21"/>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A129" s="23">
+        <f t="shared" si="2"/>
+        <v>17</v>
+      </c>
+      <c r="B129" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="C129" s="21"/>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A130" s="23">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="B130" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="C130" s="21"/>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A131" s="23">
+        <f t="shared" si="2"/>
+        <v>19</v>
+      </c>
+      <c r="B131" s="24" t="s">
+        <v>287</v>
+      </c>
+      <c r="C131" s="21"/>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A132" s="23">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="B132" s="24" t="s">
+        <v>214</v>
+      </c>
+      <c r="C132" s="21"/>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A133" s="23">
+        <f t="shared" si="2"/>
+        <v>21</v>
+      </c>
+      <c r="B133" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="C133" s="21"/>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A134" s="23">
+        <f t="shared" si="2"/>
+        <v>22</v>
+      </c>
+      <c r="B134" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="C134" s="21"/>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A135" s="23">
+        <f t="shared" si="2"/>
+        <v>23</v>
+      </c>
+      <c r="B135" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="C135" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A136" s="23">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="B136" s="24" t="s">
+        <v>293</v>
+      </c>
+      <c r="C136" s="24" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A137" s="23">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="B137" s="24" t="s">
+        <v>300</v>
+      </c>
+      <c r="C137" s="24"/>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A138" s="23">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="B138" s="24" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A139" s="23">
+        <f t="shared" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="B139" s="24" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A140" s="23">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="B140" s="24" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A141" s="23">
+        <f t="shared" si="2"/>
+        <v>29</v>
+      </c>
+      <c r="B141" s="24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A142" s="23">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="B142" s="24" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A143" s="23">
+        <f t="shared" si="2"/>
+        <v>31</v>
+      </c>
+      <c r="B143" s="24" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A144" s="23">
+        <f t="shared" si="2"/>
+        <v>32</v>
+      </c>
+      <c r="B144" s="24" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A145" s="23">
+        <f t="shared" si="2"/>
+        <v>33</v>
+      </c>
+      <c r="B145" s="24" t="s">
+        <v>304</v>
+      </c>
+      <c r="C145" s="24" t="s">
+        <v>106</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:I106" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -5436,7 +5856,7 @@
         <v>114</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D21" s="12">
         <v>2</v>

</xml_diff>